<commit_message>
add cafe sales dashboard
</commit_message>
<xml_diff>
--- a/Data_analysis_using_excel/Multiple_data_sheets.xlsx
+++ b/Data_analysis_using_excel/Multiple_data_sheets.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VISHWAS SHARMA\Documents\Xcel_portfolio\Data_analysis_using_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B39E545F-5203-4B13-8605-984072E10E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB0C7CB6-DF93-467E-BD0A-1A91BCDD771E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="8" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sales Table" sheetId="1" r:id="rId1"/>
@@ -24,8 +24,8 @@
     <sheet name="student_table(1)" sheetId="8" r:id="rId9"/>
     <sheet name="student Table" sheetId="9" r:id="rId10"/>
     <sheet name="EMI" sheetId="13" r:id="rId11"/>
-    <sheet name="Sheet2" sheetId="14" r:id="rId12"/>
-    <sheet name="Sheet3" sheetId="15" r:id="rId13"/>
+    <sheet name="Home Loan" sheetId="14" r:id="rId12"/>
+    <sheet name="Basic functions" sheetId="15" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -9368,7 +9368,7 @@
       </c>
       <c r="D15" s="77">
         <f ca="1">TODAY()</f>
-        <v>46252</v>
+        <v>46256</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -9377,7 +9377,7 @@
       </c>
       <c r="D16" s="78">
         <f ca="1">NOW()</f>
-        <v>46252.504138773147</v>
+        <v>46256.566698379633</v>
       </c>
     </row>
     <row r="17" spans="3:4" x14ac:dyDescent="0.25">
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D21" s="77">
         <f ca="1">DATEDIF(D17,D15,"d")</f>
-        <v>7306</v>
+        <v>7310</v>
       </c>
     </row>
   </sheetData>

</xml_diff>